<commit_message>
Push outputs from CI/CD (2025-07-21 23:08:18)
</commit_message>
<xml_diff>
--- a/production/Manufacturing/Assembly/BeeLight-bom.xlsx
+++ b/production/Manufacturing/Assembly/BeeLight-bom.xlsx
@@ -257,7 +257,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>38177 Auf Lager</t>
+          <t>37919 Auf Lager</t>
         </r>
       </text>
     </comment>
@@ -273,15 +273,15 @@
           <t>Qty/Price Breaks (EUR):
   Qty  -  Unit€  -  Ext€
 ================
-     1   €0.39      €0.39
-    10   €0.35      €3.52
-    25   €0.32      €8.00
-   100   €0.29     €29.20
-   250   €0.28     €70.75
-   500   €0.26    €128.50
-  1000   €0.24    €242.00
-  2500   €0.23    €562.50
-  5000   €0.21  €1,050.00</t>
+     1   €0.37      €0.37
+    10   €0.34      €3.36
+    25   €0.31      €7.65
+   100   €0.28     €27.90
+   250   €0.27     €67.50
+   500   €0.24    €122.50
+  1000   €0.23    €231.00
+  2500   €0.21    €537.50
+  5000   €0.20  €1,000.00</t>
         </r>
       </text>
     </comment>
@@ -307,7 +307,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>199028 Auf Lager</t>
+          <t>160824 Auf Lager</t>
         </r>
       </text>
     </comment>
@@ -324,14 +324,14 @@
   Qty  -  Unit€  -  Ext€
 ================
      1   €0.09      €0.09
-    10   €0.04      €0.36
-   100   €0.02      €2.20
-   500   €0.02      €8.50
+    10   €0.03      €0.34
+   100   €0.02      €2.10
+   500   €0.02      €8.00
   1000   €0.01     €15.00
   2500   €0.01     €35.00
- 10000   €0.01    €120.00
- 25000   €0.01    €275.00
- 50000   €0.01    €500.00</t>
+ 10000   €0.01    €110.00
+ 25000   €0.01    €250.00
+ 50000   €0.01    €450.00</t>
         </r>
       </text>
     </comment>
@@ -357,7 +357,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>8410 Auf Lager</t>
+          <t>8409 Auf Lager</t>
         </r>
       </text>
     </comment>
@@ -373,15 +373,15 @@
           <t>Qty/Price Breaks (EUR):
   Qty  -  Unit€  -  Ext€
 ================
-     1   €1.08      €1.08
-    10   €0.76      €7.61
-   100   €0.57     €56.80
-   500   €0.48    €241.00
-  1000   €0.45    €453.00
-  2000   €0.43    €858.00
-  4000   €0.39  €1,564.00
-  8000   €0.37  €2,976.00
- 24000   €0.37  €8,856.00</t>
+     1   €1.03      €1.03
+    10   €0.73      €7.28
+   100   €0.54     €54.30
+   500   €0.46    €230.00
+  1000   €0.43    €433.00
+  2000   €0.41    €820.00
+  4000   €0.37  €1,492.00
+  8000   €0.35  €2,840.00
+ 24000   €0.35  €8,472.00</t>
         </r>
       </text>
     </comment>
@@ -407,7 +407,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>51739 Auf Lager</t>
+          <t>51714 Auf Lager</t>
         </r>
       </text>
     </comment>
@@ -423,14 +423,14 @@
           <t>Qty/Price Breaks (EUR):
   Qty  -  Unit€  -  Ext€
 ================
-     1   €0.88      €0.88
-    10   €0.74      €7.45
-   100   €0.71     €71.30
-   500   €0.65    €323.50
-  1000   €0.62    €623.00
-  2500   €0.59  €1,482.50
-  5000   €0.56  €2,815.00
- 10000   €0.54  €5,430.00</t>
+     1   €0.84      €0.84
+    10   €0.71      €7.12
+   100   €0.68     €68.10
+   500   €0.62    €309.00
+  1000   €0.59    €595.00
+  2500   €0.57  €1,417.50
+  5000   €0.54  €2,690.00
+ 10000   €0.52  €5,190.00</t>
         </r>
       </text>
     </comment>
@@ -456,7 +456,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>3504 Auf Lager</t>
+          <t>7917 Auf Lager</t>
         </r>
       </text>
     </comment>
@@ -472,15 +472,16 @@
           <t>Qty/Price Breaks (EUR):
   Qty  -  Unit€  -  Ext€
 ================
-     1   €7.79      €7.79
-     5   €7.04     €35.20
-    10   €6.76     €67.60
-    25   €6.43    €160.75
-    50   €6.20    €310.00
-   100   €5.99    €599.00
-   500   €5.57  €2,785.00
-  1000   €5.41  €5,410.00
-  6000   €5.41 €32,460.00</t>
+     1   €7.44      €7.44
+     5   €6.73     €33.65
+    10   €6.46     €64.60
+    25   €6.14    €153.50
+    50   €5.93    €296.50
+   100   €5.73    €573.00
+   250   €5.72  €1,430.00
+   500   €5.45  €2,725.00
+  1000   €4.96  €4,960.00
+  6000   €4.96 €29,760.00</t>
         </r>
       </text>
     </comment>
@@ -506,7 +507,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>731 Auf Lager</t>
+          <t>686 Auf Lager</t>
         </r>
       </text>
     </comment>
@@ -522,8 +523,8 @@
           <t>Qty/Price Breaks (EUR):
   Qty  -  Unit€  -  Ext€
 ================
-     1   €3.83      €3.83
-  1000   €3.72  €3,720.00</t>
+     1   €3.66      €3.66
+  1000   €3.55  €3,550.00</t>
         </r>
       </text>
     </comment>
@@ -549,7 +550,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>88576 Auf Lager</t>
+          <t>98416 Auf Lager</t>
         </r>
       </text>
     </comment>
@@ -565,15 +566,15 @@
           <t>Qty/Price Breaks (EUR):
   Qty  -  Unit€  -  Ext€
 ================
-     1   €0.41      €0.41
-    10   €0.27      €2.66
-   100   €0.19     €18.60
-   500   €0.17     €83.50
-  1000   €0.14    €139.00
-  3000   €0.13    €378.00
-  6000   €0.11    €684.00
-  9000   €0.10    €900.00
- 24000   €0.10  €2,304.00</t>
+     1   €0.42      €0.42
+    10   €0.26      €2.55
+   100   €0.18     €17.80
+   500   €0.16     €79.50
+  1000   €0.14    €142.00
+  3000   €0.12    €363.00
+  6000   €0.11    €660.00
+  9000   €0.10    €855.00
+ 24000   €0.09  €2,184.00</t>
         </r>
       </text>
     </comment>
@@ -599,7 +600,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>309346 Auf Lager</t>
+          <t>300505 Auf Lager</t>
         </r>
       </text>
     </comment>
@@ -617,12 +618,12 @@
 ================
      1   €0.09      €0.09
     10   €0.02      €0.20
-   100   €0.02      €1.60
-   500   €0.01      €5.50
-  1000   €0.01     €10.00
+   100   €0.01      €1.50
+   500   €0.01      €5.00
+  1000   €0.01      €9.00
   5000   €0.01     €30.00
  10000   €0.01     €50.00
- 50000   €0.00    €200.00</t>
+ 25000   €0.00    €100.00</t>
         </r>
       </text>
     </comment>
@@ -648,11 +649,58 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>1968670 Auf Lager</t>
+          <t>1968140 Auf Lager</t>
         </r>
       </text>
     </comment>
     <comment ref="K19" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Qty/Price Breaks (EUR):
+  Qty  -  Unit€  -  Ext€
+================
+     1   €0.09      €0.09
+    10   €0.01      €0.07
+   100   €0.01      €0.50
+   500   €0.00      €1.50
+ 10000   €0.00     €20.00
+ 20000   €0.00     €20.00</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N19" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Desc: Dickfilmwiderstände - SMD 220 OHM 5%</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I20" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>96448 Auf Lager</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K20" authorId="0">
       <text>
         <r>
           <rPr>
@@ -666,41 +714,139 @@
 ================
      1   €0.09      €0.09
     10   €0.01      €0.06
-   100   €0.01      €0.50
-   500   €0.00      €2.00
+   100   €0.00      €0.40
   1000   €0.00      €3.00
- 10000   €0.00     €20.00
- 20000   €0.00     €20.00</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N19" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Desc: Dickfilmwiderstände - SMD 220 OHM 5%</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I20" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>127793 Auf Lager</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K20" authorId="0">
+ 10000   €0.00     €20.00</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N20" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Desc: Dickfilmwiderstände - SMD 1.8 kOhms 62.5mW 0402 1%</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I21" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>18873 Auf Lager</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K21" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Qty/Price Breaks (EUR):
+  Qty  -  Unit€  -  Ext€
+================
+     1   €0.14      €0.14
+    10   €0.09      €0.92
+    50   €0.08      €3.85
+   100   €0.07      €7.40
+   500   €0.06     €30.00
+  1000   €0.06     €56.00
+  2000   €0.05    €108.00
+  5000   €0.05    €230.00
+ 10000   €0.04    €380.00</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N21" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Desc: Dünnfilmwiderstände - SMD 1/16W 2.2K ohm .1% 25ppm</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I22" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>1920 Auf Lager</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K22" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Qty/Price Breaks (EUR):
+  Qty  -  Unit€  -  Ext€
+================
+     1   €0.15      €0.15
+    10   €0.10      €1.01
+    50   €0.08      €4.20
+   100   €0.08      €7.60
+   500   €0.06     €29.00
+  1000   €0.05     €52.00
+  2000   €0.05    €102.00
+  5000   €0.04    €210.00
+ 10000   €0.04    €380.00</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N22" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Desc: Dünnfilmwiderstände - SMD 1/16W 8.2K ohm .1% 25ppm</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I23" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>662189 Auf Lager</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K23" authorId="0">
       <text>
         <r>
           <rPr>
@@ -713,40 +859,41 @@
   Qty  -  Unit€  -  Ext€
 ================
      1   €0.09      €0.09
-    10   €0.01      €0.06
-   100   €0.01      €0.50
+    10   €0.01      €0.09
+   100   €0.01      €0.80
   1000   €0.00      €4.00
- 10000   €0.00     €10.00</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N20" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Desc: Dickfilmwiderstände - SMD 1.8 kOhms 62.5mW 0402 1%</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I21" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>19935 Auf Lager</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K21" authorId="0">
+  2500   €0.00      €7.50
+ 10000   €0.00     €20.00</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N23" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Desc: Dickfilmwiderstände - SMD 100 kOhms 62.5mW 0402 1%</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I24" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>4566 Auf Lager</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K24" authorId="0">
       <text>
         <r>
           <rPr>
@@ -758,158 +905,13 @@
           <t>Qty/Price Breaks (EUR):
   Qty  -  Unit€  -  Ext€
 ================
-     1   €0.14      €0.14
-    10   €0.10      €0.95
-    50   €0.08      €4.05
-   100   €0.08      €7.60
-   500   €0.06     €31.00
-  1000   €0.05     €54.00
-  5000   €0.04    €210.00
- 10000   €0.04    €390.00</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N21" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Desc: Dünnfilmwiderstände - SMD 1/16W 2.2K ohm .1% 25ppm</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I22" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>755 Auf Lager</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K22" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Qty/Price Breaks (EUR):
-  Qty  -  Unit€  -  Ext€
-================
-     1   €0.16      €0.16
-    10   €0.11      €1.12
-    50   €0.09      €4.45
-   100   €0.08      €8.00
-   500   €0.06     €31.00
-  1000   €0.06     €59.00
-  2000   €0.05    €106.00
-  5000   €0.05    €245.00
- 10000   €0.05    €470.00</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N22" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Desc: Dünnfilmwiderstände - SMD 1/16W 8.2K ohm .1% 25ppm</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I23" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>1424586 Auf Lager</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K23" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Qty/Price Breaks (EUR):
-  Qty  -  Unit€  -  Ext€
-================
-     1   €0.09      €0.09
-    10   €0.01      €0.08
-   100   €0.01      €0.60
-  1000   €0.01      €5.00
- 10000   €0.00     €10.00</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N23" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Desc: Dickfilmwiderstände - SMD 100 kOhms 62.5mW 0402 1%</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I24" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>2349 Auf Lager</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K24" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Qty/Price Breaks (EUR):
-  Qty  -  Unit€  -  Ext€
-================
-     1   €0.48      €0.48
-    10   €0.47      €4.73
-    50   €0.44     €21.95
-   100   €0.40     €40.00
-   250   €0.36     €90.00
-   400   €0.33    €130.40
-   800   €0.28    €227.20</t>
+     1   €0.46      €0.46
+    10   €0.45      €4.52
+    50   €0.42     €21.00
+   100   €0.38     €38.20
+   250   €0.34     €86.00
+   400   €0.31    €124.40
+   800   €0.27    €216.80</t>
         </r>
       </text>
     </comment>
@@ -1212,7 +1214,7 @@
     <t>11</t>
   </si>
   <si>
-    <t>R104 R105 R106</t>
+    <t>R104 R105</t>
   </si>
   <si>
     <t>1k8</t>
@@ -1338,7 +1340,7 @@
     <t>Component Count:</t>
   </si>
   <si>
-    <t>21 (21 SMD/ 0 THT)</t>
+    <t>20 (20 SMD/ 0 THT)</t>
   </si>
   <si>
     <t>Fitted Components:</t>
@@ -1449,7 +1451,7 @@
     <t>Created:</t>
   </si>
   <si>
-    <t>2025-06-29 08:57:59</t>
+    <t>2025-07-21 23:13:40</t>
   </si>
   <si>
     <t>KiCost® v1.1.20 + KiBot v1.8.4</t>
@@ -2289,7 +2291,7 @@
         <v>125</v>
       </c>
       <c r="D6" s="3">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2616,7 +2618,7 @@
         <v>79</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>80</v>
@@ -2841,7 +2843,7 @@
       </c>
       <c r="H3" s="14">
         <f>TotalCost/BoardQty</f>
-        <v>18.8984</v>
+        <v>17.9252</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -2856,11 +2858,11 @@
       </c>
       <c r="H4" s="15">
         <f>SUM(H10:H24)</f>
-        <v>18.8984</v>
+        <v>17.9252</v>
       </c>
       <c r="M4" s="15">
         <f>SUM(M10:M24)</f>
-        <v>18.8984</v>
+        <v>17.9252</v>
       </c>
       <c r="N4" s="16" t="str">
         <f>(COUNTA(M10:M24)&amp;" of "&amp;ROWS(M10:M24)&amp;" parts found")</f>
@@ -2969,26 +2971,26 @@
       </c>
       <c r="G10" s="21">
         <f>IF(MIN(K10)&lt;&gt;0,MIN(K10),"")</f>
-        <v>0.45294480000000004</v>
+        <v>0.43167900000000003</v>
       </c>
       <c r="H10" s="22">
         <f>IF(AND(ISNUMBER(F10),ISNUMBER(G10)),F10*G10,"")</f>
-        <v>0.4529</v>
+        <v>0.4317</v>
       </c>
       <c r="I10" s="20">
-        <v>38177</v>
+        <v>37919</v>
       </c>
       <c r="J10" s="20"/>
       <c r="K10" s="21">
-        <f>IFERROR(IF(OR(J10&gt;=L10,F10&gt;=L10),USD_EUR*LOOKUP(IF(J10="",F10,J10),{0,1,10,25,100,250,500,1000,2500,5000},{0.0,0.387,0.352,0.32,0.292,0.283,0.257,0.242,0.225,0.21}),"MOQ="&amp;L10),"")</f>
-        <v>0.45294480000000004</v>
+        <f>IFERROR(IF(OR(J10&gt;=L10,F10&gt;=L10),USD_EUR*LOOKUP(IF(J10="",F10,J10),{0,1,10,25,100,250,500,1000,2500,5000},{0.0,0.37,0.336,0.306,0.279,0.27,0.245,0.231,0.215,0.2}),"MOQ="&amp;L10),"")</f>
+        <v>0.43167900000000003</v>
       </c>
       <c r="L10" s="20">
         <v>1</v>
       </c>
       <c r="M10" s="22">
         <f>IFERROR(IF(J10="",F10,J10)*K10,"")</f>
-        <v>0.4529</v>
+        <v>0.4317</v>
       </c>
       <c r="N10" s="20" t="s">
         <v>137</v>
@@ -3045,26 +3047,26 @@
       </c>
       <c r="G12" s="21">
         <f>IF(MIN(K12)&lt;&gt;0,MIN(K12),"")</f>
-        <v>0.105336</v>
+        <v>0.1003362</v>
       </c>
       <c r="H12" s="22">
         <f>IF(AND(ISNUMBER(F12),ISNUMBER(G12)),F12*G12,"")</f>
-        <v>0.5267</v>
+        <v>0.5017</v>
       </c>
       <c r="I12" s="20">
-        <v>199028</v>
+        <v>160824</v>
       </c>
       <c r="J12" s="20"/>
       <c r="K12" s="21">
-        <f>IFERROR(IF(OR(J12&gt;=L12,F12&gt;=L12),USD_EUR*LOOKUP(IF(J12="",F12,J12),{0,1,10,100,500,1000,2500,10000,25000,50000},{0.0,0.09,0.036,0.022,0.017,0.015,0.014,0.012,0.011,0.01}),"MOQ="&amp;L12),"")</f>
-        <v>0.105336</v>
+        <f>IFERROR(IF(OR(J12&gt;=L12,F12&gt;=L12),USD_EUR*LOOKUP(IF(J12="",F12,J12),{0,1,10,100,500,1000,2500,10000,25000,50000},{0.0,0.086,0.034,0.021,0.016,0.015,0.014,0.011,0.01,0.009}),"MOQ="&amp;L12),"")</f>
+        <v>0.1003362</v>
       </c>
       <c r="L12" s="20">
         <v>1</v>
       </c>
       <c r="M12" s="22">
         <f>IFERROR(IF(J12="",F12,J12)*K12,"")</f>
-        <v>0.5267</v>
+        <v>0.5017</v>
       </c>
       <c r="N12" s="20" t="s">
         <v>138</v>
@@ -3092,26 +3094,26 @@
       </c>
       <c r="G13" s="21">
         <f>IF(MIN(K13)&lt;&gt;0,MIN(K13),"")</f>
-        <v>1.2640320000000003</v>
+        <v>1.2017010000000001</v>
       </c>
       <c r="H13" s="22">
         <f>IF(AND(ISNUMBER(F13),ISNUMBER(G13)),F13*G13,"")</f>
-        <v>1.264</v>
+        <v>1.2017</v>
       </c>
       <c r="I13" s="20">
-        <v>8410</v>
+        <v>8409</v>
       </c>
       <c r="J13" s="20"/>
       <c r="K13" s="21">
-        <f>IFERROR(IF(OR(J13&gt;=L13,F13&gt;=L13),USD_EUR*LOOKUP(IF(J13="",F13,J13),{0,1,10,100,500,1000,2000,4000,8000,24000},{0.0,1.08,0.761,0.568,0.482,0.453,0.429,0.391,0.372,0.369}),"MOQ="&amp;L13),"")</f>
-        <v>1.2640320000000003</v>
+        <f>IFERROR(IF(OR(J13&gt;=L13,F13&gt;=L13),USD_EUR*LOOKUP(IF(J13="",F13,J13),{0,1,10,100,500,1000,2000,4000,8000,24000},{0.0,1.03,0.728,0.543,0.46,0.433,0.41,0.373,0.355,0.353}),"MOQ="&amp;L13),"")</f>
+        <v>1.2017010000000001</v>
       </c>
       <c r="L13" s="20">
         <v>1</v>
       </c>
       <c r="M13" s="22">
         <f>IFERROR(IF(J13="",F13,J13)*K13,"")</f>
-        <v>1.264</v>
+        <v>1.2017</v>
       </c>
       <c r="N13" s="20" t="s">
         <v>139</v>
@@ -3139,26 +3141,26 @@
       </c>
       <c r="G14" s="21">
         <f>IF(MIN(K14)&lt;&gt;0,MIN(K14),"")</f>
-        <v>1.0322928</v>
+        <v>0.9835281</v>
       </c>
       <c r="H14" s="22">
         <f>IF(AND(ISNUMBER(F14),ISNUMBER(G14)),F14*G14,"")</f>
-        <v>1.0323</v>
+        <v>0.9835</v>
       </c>
       <c r="I14" s="20">
-        <v>51739</v>
+        <v>51714</v>
       </c>
       <c r="J14" s="20"/>
       <c r="K14" s="21">
-        <f>IFERROR(IF(OR(J14&gt;=L14,F14&gt;=L14),USD_EUR*LOOKUP(IF(J14="",F14,J14),{0,1,10,100,500,1000,2500,5000,10000},{0.0,0.882,0.745,0.713,0.647,0.623,0.593,0.563,0.543}),"MOQ="&amp;L14),"")</f>
-        <v>1.0322928</v>
+        <f>IFERROR(IF(OR(J14&gt;=L14,F14&gt;=L14),USD_EUR*LOOKUP(IF(J14="",F14,J14),{0,1,10,100,500,1000,2500,5000,10000},{0.0,0.843,0.712,0.681,0.618,0.595,0.567,0.538,0.519}),"MOQ="&amp;L14),"")</f>
+        <v>0.9835281</v>
       </c>
       <c r="L14" s="20">
         <v>1</v>
       </c>
       <c r="M14" s="22">
         <f>IFERROR(IF(J14="",F14,J14)*K14,"")</f>
-        <v>1.0323</v>
+        <v>0.9835</v>
       </c>
       <c r="N14" s="20" t="s">
         <v>140</v>
@@ -3186,26 +3188,26 @@
       </c>
       <c r="G15" s="21">
         <f>IF(MIN(K15)&lt;&gt;0,MIN(K15),"")</f>
-        <v>9.117416</v>
+        <v>8.680248</v>
       </c>
       <c r="H15" s="22">
         <f>IF(AND(ISNUMBER(F15),ISNUMBER(G15)),F15*G15,"")</f>
-        <v>9.1174</v>
+        <v>8.6802</v>
       </c>
       <c r="I15" s="20">
-        <v>3504</v>
+        <v>7917</v>
       </c>
       <c r="J15" s="20"/>
       <c r="K15" s="21">
-        <f>IFERROR(IF(OR(J15&gt;=L15,F15&gt;=L15),USD_EUR*LOOKUP(IF(J15="",F15,J15),{0,1,5,10,25,50,100,500,1000,6000},{0.0,7.79,7.04,6.76,6.43,6.2,5.99,5.57,5.41,5.41}),"MOQ="&amp;L15),"")</f>
-        <v>9.117416</v>
+        <f>IFERROR(IF(OR(J15&gt;=L15,F15&gt;=L15),USD_EUR*LOOKUP(IF(J15="",F15,J15),{0,1,5,10,25,50,100,250,500,1000,6000},{0.0,7.44,6.73,6.46,6.14,5.93,5.73,5.72,5.45,4.96,4.96}),"MOQ="&amp;L15),"")</f>
+        <v>8.680248</v>
       </c>
       <c r="L15" s="20">
         <v>1</v>
       </c>
       <c r="M15" s="22">
         <f>IFERROR(IF(J15="",F15,J15)*K15,"")</f>
-        <v>9.1174</v>
+        <v>8.6802</v>
       </c>
       <c r="N15" s="20" t="s">
         <v>141</v>
@@ -3233,26 +3235,26 @@
       </c>
       <c r="G16" s="21">
         <f>IF(MIN(K16)&lt;&gt;0,MIN(K16),"")</f>
-        <v>4.482632000000001</v>
+        <v>4.270122000000001</v>
       </c>
       <c r="H16" s="22">
         <f>IF(AND(ISNUMBER(F16),ISNUMBER(G16)),F16*G16,"")</f>
-        <v>4.4826</v>
+        <v>4.2701</v>
       </c>
       <c r="I16" s="20">
-        <v>731</v>
+        <v>686</v>
       </c>
       <c r="J16" s="20"/>
       <c r="K16" s="21">
-        <f>IFERROR(IF(OR(J16&gt;=L16,F16&gt;=L16),USD_EUR*LOOKUP(IF(J16="",F16,J16),{0,1,1000},{0.0,3.83,3.72}),"MOQ="&amp;L16),"")</f>
-        <v>4.482632000000001</v>
+        <f>IFERROR(IF(OR(J16&gt;=L16,F16&gt;=L16),USD_EUR*LOOKUP(IF(J16="",F16,J16),{0,1,1000},{0.0,3.66,3.55}),"MOQ="&amp;L16),"")</f>
+        <v>4.270122000000001</v>
       </c>
       <c r="L16" s="20">
         <v>1</v>
       </c>
       <c r="M16" s="22">
         <f>IFERROR(IF(J16="",F16,J16)*K16,"")</f>
-        <v>4.4826</v>
+        <v>4.2701</v>
       </c>
       <c r="N16" s="20" t="s">
         <v>142</v>
@@ -3280,26 +3282,26 @@
       </c>
       <c r="G17" s="21">
         <f>IF(MIN(K17)&lt;&gt;0,MIN(K17),"")</f>
-        <v>0.4740120000000001</v>
+        <v>0.4911807</v>
       </c>
       <c r="H17" s="22">
         <f>IF(AND(ISNUMBER(F17),ISNUMBER(G17)),F17*G17,"")</f>
-        <v>0.474</v>
+        <v>0.4912</v>
       </c>
       <c r="I17" s="20">
-        <v>88576</v>
+        <v>98416</v>
       </c>
       <c r="J17" s="20"/>
       <c r="K17" s="21">
-        <f>IFERROR(IF(OR(J17&gt;=L17,F17&gt;=L17),USD_EUR*LOOKUP(IF(J17="",F17,J17),{0,1,10,100,500,1000,3000,6000,9000,24000},{0.0,0.405,0.266,0.186,0.167,0.139,0.126,0.114,0.1,0.096}),"MOQ="&amp;L17),"")</f>
-        <v>0.4740120000000001</v>
+        <f>IFERROR(IF(OR(J17&gt;=L17,F17&gt;=L17),USD_EUR*LOOKUP(IF(J17="",F17,J17),{0,1,10,100,500,1000,3000,6000,9000,24000},{0.0,0.421,0.255,0.178,0.159,0.142,0.121,0.11,0.095,0.091}),"MOQ="&amp;L17),"")</f>
+        <v>0.4911807</v>
       </c>
       <c r="L17" s="20">
         <v>1</v>
       </c>
       <c r="M17" s="22">
         <f>IFERROR(IF(J17="",F17,J17)*K17,"")</f>
-        <v>0.474</v>
+        <v>0.4912</v>
       </c>
       <c r="N17" s="20" t="s">
         <v>143</v>
@@ -3327,26 +3329,26 @@
       </c>
       <c r="G18" s="21">
         <f>IF(MIN(K18)&lt;&gt;0,MIN(K18),"")</f>
-        <v>0.105336</v>
+        <v>0.1003362</v>
       </c>
       <c r="H18" s="22">
         <f>IF(AND(ISNUMBER(F18),ISNUMBER(G18)),F18*G18,"")</f>
-        <v>0.1053</v>
+        <v>0.1003</v>
       </c>
       <c r="I18" s="20">
-        <v>309346</v>
+        <v>300505</v>
       </c>
       <c r="J18" s="20"/>
       <c r="K18" s="21">
-        <f>IFERROR(IF(OR(J18&gt;=L18,F18&gt;=L18),USD_EUR*LOOKUP(IF(J18="",F18,J18),{0,1,10,100,500,1000,5000,10000,50000},{0.0,0.09,0.02,0.016,0.011,0.01,0.006,0.005,0.004}),"MOQ="&amp;L18),"")</f>
-        <v>0.105336</v>
+        <f>IFERROR(IF(OR(J18&gt;=L18,F18&gt;=L18),USD_EUR*LOOKUP(IF(J18="",F18,J18),{0,1,10,100,500,1000,5000,10000,25000},{0.0,0.086,0.02,0.015,0.01,0.009,0.006,0.005,0.004}),"MOQ="&amp;L18),"")</f>
+        <v>0.1003362</v>
       </c>
       <c r="L18" s="20">
         <v>1</v>
       </c>
       <c r="M18" s="22">
         <f>IFERROR(IF(J18="",F18,J18)*K18,"")</f>
-        <v>0.1053</v>
+        <v>0.1003</v>
       </c>
       <c r="N18" s="20" t="s">
         <v>144</v>
@@ -3374,26 +3376,26 @@
       </c>
       <c r="G19" s="21">
         <f>IF(MIN(K19)&lt;&gt;0,MIN(K19),"")</f>
-        <v>0.105336</v>
+        <v>0.1003362</v>
       </c>
       <c r="H19" s="22">
         <f>IF(AND(ISNUMBER(F19),ISNUMBER(G19)),F19*G19,"")</f>
-        <v>0.1053</v>
+        <v>0.1003</v>
       </c>
       <c r="I19" s="20">
-        <v>1968670</v>
+        <v>1968140</v>
       </c>
       <c r="J19" s="20"/>
       <c r="K19" s="21">
-        <f>IFERROR(IF(OR(J19&gt;=L19,F19&gt;=L19),USD_EUR*LOOKUP(IF(J19="",F19,J19),{0,1,10,100,500,1000,10000,20000},{0.0,0.09,0.006,0.005,0.004,0.003,0.002,0.001}),"MOQ="&amp;L19),"")</f>
-        <v>0.105336</v>
+        <f>IFERROR(IF(OR(J19&gt;=L19,F19&gt;=L19),USD_EUR*LOOKUP(IF(J19="",F19,J19),{0,1,10,100,500,10000,20000},{0.0,0.086,0.007,0.005,0.003,0.002,0.001}),"MOQ="&amp;L19),"")</f>
+        <v>0.1003362</v>
       </c>
       <c r="L19" s="20">
         <v>1</v>
       </c>
       <c r="M19" s="22">
         <f>IFERROR(IF(J19="",F19,J19)*K19,"")</f>
-        <v>0.1053</v>
+        <v>0.1003</v>
       </c>
       <c r="N19" s="20" t="s">
         <v>145</v>
@@ -3416,31 +3418,31 @@
         <v>84</v>
       </c>
       <c r="F20" s="20">
-        <f>CEILING(BoardQty*3,1)</f>
-        <v>3</v>
+        <f>CEILING(BoardQty*2,1)</f>
+        <v>2</v>
       </c>
       <c r="G20" s="21">
         <f>IF(MIN(K20)&lt;&gt;0,MIN(K20),"")</f>
-        <v>0.105336</v>
+        <v>0.1003362</v>
       </c>
       <c r="H20" s="22">
         <f>IF(AND(ISNUMBER(F20),ISNUMBER(G20)),F20*G20,"")</f>
-        <v>0.316</v>
+        <v>0.2007</v>
       </c>
       <c r="I20" s="20">
-        <v>127793</v>
+        <v>96448</v>
       </c>
       <c r="J20" s="20"/>
       <c r="K20" s="21">
-        <f>IFERROR(IF(OR(J20&gt;=L20,F20&gt;=L20),USD_EUR*LOOKUP(IF(J20="",F20,J20),{0,1,10,100,1000,10000},{0.0,0.09,0.006,0.005,0.004,0.001}),"MOQ="&amp;L20),"")</f>
-        <v>0.105336</v>
+        <f>IFERROR(IF(OR(J20&gt;=L20,F20&gt;=L20),USD_EUR*LOOKUP(IF(J20="",F20,J20),{0,1,10,100,1000,10000},{0.0,0.086,0.006,0.004,0.003,0.002}),"MOQ="&amp;L20),"")</f>
+        <v>0.1003362</v>
       </c>
       <c r="L20" s="20">
         <v>1</v>
       </c>
       <c r="M20" s="22">
         <f>IFERROR(IF(J20="",F20,J20)*K20,"")</f>
-        <v>0.316</v>
+        <v>0.2007</v>
       </c>
       <c r="N20" s="20" t="s">
         <v>146</v>
@@ -3468,26 +3470,26 @@
       </c>
       <c r="G21" s="21">
         <f>IF(MIN(K21)&lt;&gt;0,MIN(K21),"")</f>
-        <v>0.1685376</v>
+        <v>0.16100460000000003</v>
       </c>
       <c r="H21" s="22">
         <f>IF(AND(ISNUMBER(F21),ISNUMBER(G21)),F21*G21,"")</f>
-        <v>0.1685</v>
+        <v>0.161</v>
       </c>
       <c r="I21" s="20">
-        <v>19935</v>
+        <v>18873</v>
       </c>
       <c r="J21" s="20"/>
       <c r="K21" s="21">
-        <f>IFERROR(IF(OR(J21&gt;=L21,F21&gt;=L21),USD_EUR*LOOKUP(IF(J21="",F21,J21),{0,1,10,50,100,500,1000,5000,10000},{0.0,0.144,0.095,0.081,0.076,0.062,0.054,0.042,0.039}),"MOQ="&amp;L21),"")</f>
-        <v>0.1685376</v>
+        <f>IFERROR(IF(OR(J21&gt;=L21,F21&gt;=L21),USD_EUR*LOOKUP(IF(J21="",F21,J21),{0,1,10,50,100,500,1000,2000,5000,10000},{0.0,0.138,0.092,0.077,0.074,0.06,0.056,0.054,0.046,0.038}),"MOQ="&amp;L21),"")</f>
+        <v>0.16100460000000003</v>
       </c>
       <c r="L21" s="20">
         <v>1</v>
       </c>
       <c r="M21" s="22">
         <f>IFERROR(IF(J21="",F21,J21)*K21,"")</f>
-        <v>0.1685</v>
+        <v>0.161</v>
       </c>
       <c r="N21" s="20" t="s">
         <v>147</v>
@@ -3515,26 +3517,26 @@
       </c>
       <c r="G22" s="21">
         <f>IF(MIN(K22)&lt;&gt;0,MIN(K22),"")</f>
-        <v>0.18960480000000002</v>
+        <v>0.1703382</v>
       </c>
       <c r="H22" s="22">
         <f>IF(AND(ISNUMBER(F22),ISNUMBER(G22)),F22*G22,"")</f>
-        <v>0.1896</v>
+        <v>0.1703</v>
       </c>
       <c r="I22" s="20">
-        <v>755</v>
+        <v>1920</v>
       </c>
       <c r="J22" s="20"/>
       <c r="K22" s="21">
-        <f>IFERROR(IF(OR(J22&gt;=L22,F22&gt;=L22),USD_EUR*LOOKUP(IF(J22="",F22,J22),{0,1,10,50,100,500,1000,2000,5000,10000},{0.0,0.162,0.112,0.089,0.08,0.062,0.059,0.053,0.049,0.047}),"MOQ="&amp;L22),"")</f>
-        <v>0.18960480000000002</v>
+        <f>IFERROR(IF(OR(J22&gt;=L22,F22&gt;=L22),USD_EUR*LOOKUP(IF(J22="",F22,J22),{0,1,10,50,100,500,1000,2000,5000,10000},{0.0,0.146,0.101,0.084,0.076,0.058,0.052,0.051,0.042,0.038}),"MOQ="&amp;L22),"")</f>
+        <v>0.1703382</v>
       </c>
       <c r="L22" s="20">
         <v>1</v>
       </c>
       <c r="M22" s="22">
         <f>IFERROR(IF(J22="",F22,J22)*K22,"")</f>
-        <v>0.1896</v>
+        <v>0.1703</v>
       </c>
       <c r="N22" s="20" t="s">
         <v>148</v>
@@ -3562,26 +3564,26 @@
       </c>
       <c r="G23" s="21">
         <f>IF(MIN(K23)&lt;&gt;0,MIN(K23),"")</f>
-        <v>0.105336</v>
+        <v>0.1003362</v>
       </c>
       <c r="H23" s="22">
         <f>IF(AND(ISNUMBER(F23),ISNUMBER(G23)),F23*G23,"")</f>
-        <v>0.1053</v>
+        <v>0.1003</v>
       </c>
       <c r="I23" s="20">
-        <v>1424586</v>
+        <v>662189</v>
       </c>
       <c r="J23" s="20"/>
       <c r="K23" s="21">
-        <f>IFERROR(IF(OR(J23&gt;=L23,F23&gt;=L23),USD_EUR*LOOKUP(IF(J23="",F23,J23),{0,1,10,100,1000,10000},{0.0,0.09,0.008,0.006,0.005,0.001}),"MOQ="&amp;L23),"")</f>
-        <v>0.105336</v>
+        <f>IFERROR(IF(OR(J23&gt;=L23,F23&gt;=L23),USD_EUR*LOOKUP(IF(J23="",F23,J23),{0,1,10,100,1000,2500,10000},{0.0,0.086,0.009,0.008,0.004,0.003,0.002}),"MOQ="&amp;L23),"")</f>
+        <v>0.1003362</v>
       </c>
       <c r="L23" s="20">
         <v>1</v>
       </c>
       <c r="M23" s="22">
         <f>IFERROR(IF(J23="",F23,J23)*K23,"")</f>
-        <v>0.1053</v>
+        <v>0.1003</v>
       </c>
       <c r="N23" s="20" t="s">
         <v>149</v>
@@ -3609,26 +3611,26 @@
       </c>
       <c r="G24" s="21">
         <f>IF(MIN(K24)&lt;&gt;0,MIN(K24),"")</f>
-        <v>0.5582808</v>
+        <v>0.5320152</v>
       </c>
       <c r="H24" s="22">
         <f>IF(AND(ISNUMBER(F24),ISNUMBER(G24)),F24*G24,"")</f>
-        <v>0.5583</v>
+        <v>0.532</v>
       </c>
       <c r="I24" s="20">
-        <v>2349</v>
+        <v>4566</v>
       </c>
       <c r="J24" s="20"/>
       <c r="K24" s="21">
-        <f>IFERROR(IF(OR(J24&gt;=L24,F24&gt;=L24),USD_EUR*LOOKUP(IF(J24="",F24,J24),{0,1,10,50,100,250,400,800},{0.0,0.477,0.473,0.439,0.4,0.36,0.326,0.284}),"MOQ="&amp;L24),"")</f>
-        <v>0.5582808</v>
+        <f>IFERROR(IF(OR(J24&gt;=L24,F24&gt;=L24),USD_EUR*LOOKUP(IF(J24="",F24,J24),{0,1,10,50,100,250,400,800},{0.0,0.456,0.452,0.42,0.382,0.344,0.311,0.271}),"MOQ="&amp;L24),"")</f>
+        <v>0.5320152</v>
       </c>
       <c r="L24" s="20">
         <v>1</v>
       </c>
       <c r="M24" s="22">
         <f>IFERROR(IF(J24="",F24,J24)*K24,"")</f>
-        <v>0.5583</v>
+        <v>0.532</v>
       </c>
       <c r="N24" s="20" t="s">
         <v>150</v>
@@ -3639,7 +3641,7 @@
         <v>154</v>
       </c>
       <c r="C26">
-        <v>1.1704</v>
+        <v>1.1667</v>
       </c>
       <c r="G26" s="13" t="s">
         <v>152</v>

</xml_diff>